<commit_message>
update puma until 2022
</commit_message>
<xml_diff>
--- a/data/input/puma.xlsx
+++ b/data/input/puma.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Saowalak/Desktop/CEOCommunication/data/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A41CC91-8584-2D47-87B2-CA2201111921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{678E623C-AB8D-1C40-977D-5718C03E6851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9940" yWindow="600" windowWidth="18860" windowHeight="17400" xr2:uid="{05EFD2A9-923A-834E-A816-A8C1AAE62552}"/>
+    <workbookView xWindow="280" yWindow="600" windowWidth="28520" windowHeight="17400" activeTab="2" xr2:uid="{05EFD2A9-923A-834E-A816-A8C1AAE62552}"/>
   </bookViews>
   <sheets>
     <sheet name="2020" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="137">
   <si>
     <t>ID</t>
   </si>
@@ -247,6 +247,221 @@
   </si>
   <si>
     <t>ceo</t>
+  </si>
+  <si>
+    <t>I hope this letter finds you well despite the current challenges around the world. After more than two years, the COVID-19 pandemic still has a negative impact on our daily lives and business and now we’re also facing a conflict in the heart of Europe that is causing terrible human suffering.</t>
+  </si>
+  <si>
+    <t>We’re in constant dialogue with all our stakeholders in Ukraine and we do our utmost to support our local employees and their families as well as all our partners, ambassadors, and athletes wherever we can. Ensuring the health and safety of our people continues to be our number one priority, as we have already demonstrated throughout the COVID-19 pandemic. We have set up a safe house in Ukraine, we are delivering food, water, and other necessities directly to our people and we are helping women and children who want to leave the country. We currently have 40 women and children in accommodation in Poland and about 120 here in Germany. Many of the adults have already started working and most of the children are already attending schools and kindergarten. Their positive attitude and mindset, as well as their willingness to work and integrate, is remarkable. They are strong and positive people. I sincerely hope that this conflict will be solved diplomatically as soon as possible, that further bloodshed can be avoided and that peace will be restored.</t>
+  </si>
+  <si>
+    <t>While we are most concerned about the lives and livelihoods of the people who are directly affected in Ukraine and by the COVID-19 pandemic, the conflict as well as the pandemic also have a significant business impact on our sector and on PUMA. In addition to the impact on our operations in Russia and Ukraine, we continue to face some of the challenges that we already saw during the course of 2021: COVID-19 related lockdowns and restrictions in different parts of the world, a weak consumer sentiment in some key markets, significant challenges in our supply chain, strong inflationary pressures, and geopolitical tensions.</t>
+  </si>
+  <si>
+    <t>Despite all these challenges, 2021 was a very successful year for us. To be specific, it was the best year in PUMA’s history. Due to our continued brand momentum combined with high operational flexibility and a fantastic effort from our employees, our sales grew by 32% to EUR 6,805m and EBIT grew by 166% to EUR 557m. Compared to the pre-pandemic level of 2019, our sales increased by 30%, resulting in a two-year CAGR of around 15% during these challenging times. Our strategy of working closely together with all our suppliers and retail partners to manage short-term issues without hindering our mid-term momentum continued to pay off. Our external partners supported us in an extraordinary way and the dedication and commitment of all our employees during such a challenging year was truly exceptional. A lot of our employees went far beyond what a company can expect from them and in the name of the entire PUMA Board, I would like to thank everyone for their contribution towards making these results possible. People make the difference and our PUMA family is our biggest strength and asset.</t>
+  </si>
+  <si>
+    <t>Throughout 2021, we continued to focus on the three main areas that we defined in early 2020 in reaction to the COVID-19 pandemic: Deal with COVID, continue to drive the business and continue to do the right thing in areas such as social responsibility and environmental sustainability.</t>
+  </si>
+  <si>
+    <t>Dealing with COVID first and foremost meant ensuring the health and safety of our people and everyone in our value chain. We continued to adopt and comply with very strict health and safety measures across our operations and rolled out vaccination programs for our employees in countries where this was possible. This helped us achieve a vaccination rate of more than 90% at our headquarters in Herzogenaurach by mid-July. At the end of the year, we followed up with booster vaccinations. I would once again like to thank our People &amp; Organization teams (formerly known as Human Resources) around the world for successfully managing a second year of COVID-19 and supporting our employees in the best way possible.</t>
+  </si>
+  <si>
+    <t>Until around the first quarter 2021, the COVID-19 pandemic mainly impacted the store operations of our own retail organization and of our retail partners due to mandatory store closures and other restrictions. This was followed by significant disruptions in our supply chain due to lockdowns and factory closures in key sourcing countries such as Bangladesh, Cambodia, China and Vietnam. Especially, the lockdown in the third quarter in 2021 in the south of Vietnam, one of our most important sourcing destinations, had a very negative impact on our supply chain. Due to strict local lockdown measures, the production at our footwear, apparel and accessories suppliers in the south of Vietnam was suspended for about ten weeks, affecting approximately 15% of our global sourcing volumes. We tried to minimize delays as much as possible and shifted part of the volumes to other sourcing locations where possible. Thanks to the quick rollout of the vaccination program in the south of Vietnam, the factories gradually reopened during October and ramped up to full production by the end of year. After our suppliers resumed normal operations, we saw fewer and very localized factory closures in some parts of Asia, which did not significantly impact our product supply. We’re very thankful to our suppliers for being a part of the PUMA family. The strong collaboration, long-term partnership and all their incredible support ensured the continued supply of products under very difficult circumstances.</t>
+  </si>
+  <si>
+    <t>The COVID-19 pandemic also had a major impact on other parts of our supply chain, and we had to deal with capacity constraints, container shortages and harbor congestion in ocean freight, but also significant challenges in air freight and land-based transportation. All these constraints led to a strong increase in freight costs, which further fueled inflationary pressures, in addition to rising costs for energy, raw materials and labor.</t>
+  </si>
+  <si>
+    <t>As manifested in our strong sales growth, we also continued to drive the business in 2021. After the end of the COVID-19 related lockdowns, we witnessed a certain “normalization” of buying patterns, with more consumers shopping offline again instead of online. In our Direct-to-Consumer business, we therefore saw a higher growth rate in our brick &amp; mortar stores compared to our eCommerce sites. However, both channels grew by double-digits last year, and we continued to invest in the optimization of our store portfolio, the consumer experience on our existing sites as well as the launch of new eCommerce sites. During a time of limited supply, we continued to prioritize our retail partners in terms of product allocation. We strongly believe in a multi-brand retail environment and will therefore strengthen the relationship with all our retail partners around the world and do everything we can to service them in the best way possible.</t>
+  </si>
+  <si>
+    <t>After a year without any major sporting events in 2020, we were also excited to see sports leagues, tournaments and other competitions resume in the course of 2021, for the most part including live spectators.</t>
+  </si>
+  <si>
+    <t>The summer of 2021 was exceptional for our teams and athletes, who delivered world class performances on track and on the pitch. We underlined our credibility and high ambitions in football with the victory of the PUMA-sponsored national team Italy at UEFA Euro 2020, several league and cup titles of our PUMA-sponsored club teams and great on-pitch visibility of our products. At the Tokyo Olympics and Paralympics, our athletes won more than 70 medals, demonstrating the performance credentials of our products on the world stage, including our new NITRO running shoes that I personally am exceptionally proud of. We also continued our successful re-entry into basketball, especially for the North American market and launched our first signature shoe with LaMelo Ball at the end of the year. The strengthening of our performance credibility has always been important to us and I’m very happy about the great progress that we’ve seen across football, running, fitness, golf, motorsport, basketball and other
+locally relevant sports. In Sportstyle, we also continued to build brand heat through exciting new products and collaborations and by offering a comprehensive collection across all relevant price points, including a strong focus on comfort. We are very happy to see that our classics business is growing strongly. Our PUMA Archive is full of footwear and apparel from the 70s, 80s and 90s, for which there is currently a lot of demand in youth culture. We’re also very satisfied to see the continued momentum in our women’s business, following the launch of our “She Moves Us” brand platform, and we will keep capitalizing on our truly inclusive product offering across genders, age groups etc.!</t>
+  </si>
+  <si>
+    <t>We also continued to focus on what we call “Doing the right thing”. We want to be a good corporate citizen and embed our social responsibility and our environmental sustainability into all our business practices. With regards to social responsibility, we continued with multiple initiatives under our #REFORM platform to promote universal equality. We strongly believe that people should be treated equally irrespective of their gender, age, skin color, religious believes, sexual orientation or any other factor. Together with our brand ambassadors and partner organizations, we want to do our part to promote universal equality and fight any form of discrimination in sports and society as a whole. As part of our ambitious 10FOR25 sustainability targets, we implemented more sustainable business practices in all our business operations from sourcing to retail and further increased the usage of more sustainable materials and the overall share of more sustainable products in our collections. We also increased our focus on circularity, with several pilot projects and strengthened our consumer-facing sustainability communication through our FOREVER BETTER brand platform. I, together with my team, attended the COP26 climate conference in Glasgow to emphasize our commitment in the fight against climate change and to work towards limiting the global temperature rise to 1.5 degrees Celsius above pre-industrial levels. We have all theseinitiatives because we really believe in them, as part of PUMA’s core values, and we will continue to do the right thing.</t>
+  </si>
+  <si>
+    <t>Given our strong performance in 2021 and good momentum in the first months of 2022, we’re also optimistic for the future of our industry in general and for PUMA in particular, despite the external challenges. The underlying dynamics in our sector remain very strong given the increasing participation in sports, the ongoing sneaker trend and the continued casualization among consumers all around the world. We also see PUMA’s brand momentum continuing and we will ensure operational flexibility in an increasingly volatile and unpredictable marketplace. As we have already done during the past years, we will continue to work very closely with all our retail partners to further increase our shelf space and support the sell-through of our products in their stores. We have focused on building strong partnerships with all our key stakeholders such as suppliers, retailers, ambassadors and athletes, helping them as well as us through the ongoing challenges. We will continue to foster these partnerships in the future. We therefore expect 2022 to be another record year for PUMA, with a net sales growth of at least 10%, with upside potential, and an EBIT of EUR 600 – 700 million. The objective is not to maximize short-term EBIT, but to continue to have healthy long-term growth in both sales and EBIT. We will also keep on putting our people first and take care of all our partners.</t>
+  </si>
+  <si>
+    <t>Let’s stay positive and hope that peace in Ukraine will be restored as soon as possible and that the impact of the COVID-19 pandemic will continue to decrease.</t>
+  </si>
+  <si>
+    <t>Thank you for being part of the PUMA family!
+Stay strong, healthy and optimistic!
+Bjørn Gulden
+Chief Executive Officer PUMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">title </t>
+  </si>
+  <si>
+    <t>DEU21P01-00</t>
+  </si>
+  <si>
+    <t>DEU21P02-00</t>
+  </si>
+  <si>
+    <t>DEU21P03-00</t>
+  </si>
+  <si>
+    <t>DEU21P04-00</t>
+  </si>
+  <si>
+    <t>DEU21P05-00</t>
+  </si>
+  <si>
+    <t>DEU21P06-00</t>
+  </si>
+  <si>
+    <t>DEU21P07-00</t>
+  </si>
+  <si>
+    <t>DEU21P08-00</t>
+  </si>
+  <si>
+    <t>DEU21P09-00</t>
+  </si>
+  <si>
+    <t>DEU21P10-00</t>
+  </si>
+  <si>
+    <t>DEU21P11-00</t>
+  </si>
+  <si>
+    <t>DEU21P12-00</t>
+  </si>
+  <si>
+    <t>DEU21P13-00</t>
+  </si>
+  <si>
+    <t>DEU21P14-00</t>
+  </si>
+  <si>
+    <t>DEU21P15-00</t>
+  </si>
+  <si>
+    <t>Arne Freundt</t>
+  </si>
+  <si>
+    <t>I am honored to write this letter to you for the first time as new CEO of PUMA. I have been part of the PUMA family for more than a decade, but last year has certainly been a very special one. I feel privileged that I am now leading this company with its fantastic people to take PUMA to the next level. Let me share with you the developments and successes of 2022 and give you a brief outlook on the exciting things to come.</t>
+  </si>
+  <si>
+    <t>2022 has been the best year in PUMA's history so far! We achieved record-breaking sales and earnings. Our revenue increased by 18.9% (ca) to € 8,465 million and our operating result (EBIT) increased by 15.0% to € 640.6 million. This success was driven by our continued brand momentum and successful product launches as well as continued trustful relationships with our athletes and partners around the globe. And even more by the dedication and hard work of our incredible PUMA family.</t>
+  </si>
+  <si>
+    <t>As 2022 has brought new challenges for all of us, the PUMA Family once again proved to stand by each other. Despite repeated lockdowns that particularly affected our Chinese colleagues, our people remained dedicated to keeping ourproduction and business running smoothly. And when Russia started the war against Ukraine, we quickly set up a support program for our employees, athletes, and partners in Ukraine. Many employees have also taken initiatives themselves to support our colleagues. This makes me proud. Against this backdrop of crises, I am all the more grateful that we have managed to achieve a seamless transition in our organization and to build on the successes of the past years. On behalf of the entire Board, I would like to thank the PUMA family for this very smooth transition and for all working together every day to ensure PUMA's continued success.</t>
+  </si>
+  <si>
+    <t>Besides our strong team a huge part of the achievements was down to our partners. We continued to focus and to further deepen our partnerships along the whole value chain. Our objective is to build mutual beneficial relationships which create value and innovations and make us more resilient. Under my leadership, PUMA will continue to be the best partner for our retailers, suppliers, and athletes.</t>
+  </si>
+  <si>
+    <t>At PUMA, we also aspire not only to be the best partner, but also to make our contribution towards a more sustainable world. It is important that we continue to make steady progress towards our 10 for 25 sustainability targets. Last year, we made 70% of our products from more sustainable materials. We also achieved important milestones in sourcing and manufacturing. I am particularly proud that PUMA has been able to reduce its emissions despite its strong growth in recent years. For our progress, we have received a lot of awards last year such as Business of Fashion naming us the most sustainable brand. For us this is a great recognition and motivation to continue the journey we have embarked on.</t>
+  </si>
+  <si>
+    <t>Our brand has continued to gain momentum, thanks to our commitment to quality, innovation, and the right collaborations with leading athletes and fashion icons. We have witnessed a steady increase in customer loyalty and engagement, which is a testament to the strength of our brand and the quality of our products.</t>
+  </si>
+  <si>
+    <t>We are proud to sponsor some of the world's leading football clubs like Manchester City and AC Milan, both of whom have had exceptional seasons. Our partnership with these teams has strengthened our brand presence in the world of football and enables us to expand loyalty and affinity with the fans. We were also thrilled to see Morocco become the first African team to reach the semi-finals of the football World Cup. As a brand that values diversity and inclusivity, we were honored to have played a part in this historic moment and look forward to supporting African football in the years to come. At the World Athletics Championships in Eugene, Oregon, USA, our athletes won numerous gold medals and set new records true to our brand mantra FOREVER.FASTER.</t>
+  </si>
+  <si>
+    <t>Besides the sports arenas, we made a successful comeback at the New York Fashion Show. FUTROGRADE showcased a selection of looks - from both current and future seasons, as well as custom pieces - which were curated by PUMA Designer and Creative Director, June Ambrose. We have received great feedback from customers and influencers alike and are confident that our footprint in fashion will continue to grow and evolve.</t>
+  </si>
+  <si>
+    <t>PUMA always aims to team-up with the world’s fastest athletes and most exciting cultural icons of our times to create the best and most innovative products for our athletes and customers. That is why we have also welcomed several key new PUMA ambassadors, including world-renowned athletes like Elain Thompson-Herah, Nalyssa Smith, Emmanuel Korir, Mutaz Essa Barshim, and cultural icons like Skepta and Dixie D'Amelio. These individuals embody our brand values and vision and will inspire every athlete to achieve their goals and live their best lives. We are also proud that Sara Björk made a successful comeback to elite level football following her pregnancy while we closely accompanied her along the way.</t>
+  </si>
+  <si>
+    <t>For 75 years, PUMA has relentlessly advanced sport by creating the best products for the world's fastest athletes. In 2022, we continued to significantly improve our product offering across all business units. Our performance footwear was successful both in terms of innovation and consumer satisfaction, with the award-winning VELOCITY and DEVIATE featuring PUMA's NITRO technology. In addition to running, we saw very strong momentum in football and basketball, also driven by our great innovations, our continued high-profile collaborations and the athletic success of our brand ambassadors in last year's tournaments.</t>
+  </si>
+  <si>
+    <t>In terms of distribution and in line with our partnership strategy, we continued to focus on wholesale first. Wholesale plays a pivotal role in our strategy – not only due to their distribution reach, but also due to their retail and service excellence. I also believe that it is crucial for our consumers to have the best product offering of each brand next to each other in our wholesale partner stores. This allows our consumers to take the best purchasing decision in terms of technology, quality, design and value. I am convinced that PUMA products can compete with any competitor’s product on the shelves.</t>
+  </si>
+  <si>
+    <t>Our owned and operated brick and mortar as well as eCommerce stores are complementing our distribution mix, but we don’t have any ambition to replace wholesale partners with our Direct-to-Consumer channels. In our Direct-to-Consumer channels, we will continue to focus on storytelling to educate our consumers about the strengths and width of our brand and our products.</t>
+  </si>
+  <si>
+    <t>To achieve this objective, we optimized our retail network with new store locations and flagship stores in key markets. We also launched new web shops, extending our online reach to consumers in more than 50 countries. As part of our ongoing commitment to improve the customer experience, we launched a new shopping app for our most loyal customers in selected markets, with plans to roll it out to more markets in the coming months.</t>
+  </si>
+  <si>
+    <t>Our commitment to digitalization is not limited to our channels. As part of our ongoing efforts to modernize our infrastructure, we made significant investments in digitalizing our entire business and modernizing our offices to make our internal processes even more efficient.</t>
+  </si>
+  <si>
+    <t>2022 was a successful year. We achieved the ambitious goals we set for ourselves. But we are not leaning back and continue to be hungry to gain more market share. With the market headwinds and uncertainties in the industry, 2023 will for sure be a transition year. We continued our growth trajectory in the first quarter and recorded double-digit sales growth. For the upcoming quarters, we expect a tougher trading environment and thus a softer growth trajectory. This is fully in line with our initial guidance, and we can confirm our outlook for 2023, expecting a currency-adjusted sales growth in the high single-digit percentage range and operating result (EBIT) in a range of € 590 million to € 670 million (2022: € 641 million).</t>
+  </si>
+  <si>
+    <t>For 2023 and onwards, we will continue to focus on implementing our successful strategy and put further emphasis on three strategic priorities: elevate our brand, win in the U.S., and return to growth in China.</t>
+  </si>
+  <si>
+    <t>I would like to thank all our employees for their continued hard work and dedication to the brand and our shareholders and stakeholders for supporting us on our journey.</t>
+  </si>
+  <si>
+    <t>Together with the entire PUMA family and all our stakeholders, I look forward to continuing our exciting way ahead and achieving even greater success in the future</t>
+  </si>
+  <si>
+    <t>Arne Freundt
+Chief Executive Officer, PUMA</t>
+  </si>
+  <si>
+    <t>DEU22P01-00</t>
+  </si>
+  <si>
+    <t>DEU22P02-00</t>
+  </si>
+  <si>
+    <t>DEU22P03-00</t>
+  </si>
+  <si>
+    <t>DEU22P04-00</t>
+  </si>
+  <si>
+    <t>DEU22P05-00</t>
+  </si>
+  <si>
+    <t>DEU22P06-00</t>
+  </si>
+  <si>
+    <t>DEU22P07-00</t>
+  </si>
+  <si>
+    <t>DEU22P08-00</t>
+  </si>
+  <si>
+    <t>DEU22P09-00</t>
+  </si>
+  <si>
+    <t>DEU22P10-00</t>
+  </si>
+  <si>
+    <t>DEU22P11-00</t>
+  </si>
+  <si>
+    <t>DEU22P12-00</t>
+  </si>
+  <si>
+    <t>DEU22P13-00</t>
+  </si>
+  <si>
+    <t>DEU22P14-00</t>
+  </si>
+  <si>
+    <t>DEU22P15-00</t>
+  </si>
+  <si>
+    <t>DEU22P16-00</t>
+  </si>
+  <si>
+    <t>DEU22P17-00</t>
+  </si>
+  <si>
+    <t>DEU22P18-00</t>
+  </si>
+  <si>
+    <t>DEU22P19-00</t>
   </si>
 </sst>
 </file>
@@ -629,8 +844,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DA7F0E8F-45C6-6043-B094-E3D95B97FF2A}" name="Tableau13" displayName="Tableau13" ref="A1:N2" totalsRowShown="0" headerRowDxfId="81" dataDxfId="80">
-  <autoFilter ref="A1:N2" xr:uid="{B70DB9F7-BC01-0C48-BBE7-48DE4E59DAD7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DA7F0E8F-45C6-6043-B094-E3D95B97FF2A}" name="Tableau13" displayName="Tableau13" ref="A1:N17" totalsRowShown="0" headerRowDxfId="81" dataDxfId="80">
+  <autoFilter ref="A1:N17" xr:uid="{B70DB9F7-BC01-0C48-BBE7-48DE4E59DAD7}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N2">
     <sortCondition ref="A1:A2"/>
   </sortState>
@@ -655,8 +870,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C7C650FA-A8BE-374F-A02C-24C279A2D67A}" name="Tableau134" displayName="Tableau134" ref="A1:N2" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66">
-  <autoFilter ref="A1:N2" xr:uid="{B70DB9F7-BC01-0C48-BBE7-48DE4E59DAD7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C7C650FA-A8BE-374F-A02C-24C279A2D67A}" name="Tableau134" displayName="Tableau134" ref="A1:N21" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66">
+  <autoFilter ref="A1:N21" xr:uid="{B70DB9F7-BC01-0C48-BBE7-48DE4E59DAD7}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N2">
     <sortCondition ref="A1:A2"/>
   </sortState>
@@ -1753,11 +1968,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAD18CE3-D2D1-DD49-8602-5C2A7C693BA7}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="64.1640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="105.33203125" style="1" customWidth="1"/>
     <col min="3" max="3" width="12.5" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.83203125" style="1" customWidth="1"/>
@@ -1812,11 +2027,16 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="2"/>
+      <c r="B2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>82</v>
+      </c>
       <c r="G2" s="1" t="s">
         <v>25</v>
       </c>
@@ -1831,6 +2051,492 @@
       </c>
       <c r="K2" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="68" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J3" s="1">
+        <v>2021</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="153" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="1">
+        <v>2021</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="102" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="1">
+        <v>2021</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="153" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J6" s="1">
+        <v>2021</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="68" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J7" s="1">
+        <v>2021</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="102" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" s="1">
+        <v>2021</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="221" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J9" s="1">
+        <v>2021</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="102" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J10" s="1">
+        <v>2021</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="136" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J11" s="1">
+        <v>2021</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="34" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J12" s="1">
+        <v>2021</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M12" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="255" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J13" s="1">
+        <v>2021</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="221" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J14" s="1">
+        <v>2021</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="187" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J15" s="1">
+        <v>2021</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M15" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="34" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J16" s="1">
+        <v>2021</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L16" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M16" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="68" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J17" s="1">
+        <v>2021</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L17" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M17" s="1" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1843,11 +2549,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8482D037-842C-3D44-82D2-0DCAF2D2098B}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="64.1640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="88.83203125" style="1" customWidth="1"/>
     <col min="3" max="3" width="12.5" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.83203125" style="1" customWidth="1"/>
@@ -1902,11 +2608,16 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="2"/>
+      <c r="B2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>82</v>
+      </c>
       <c r="G2" s="1" t="s">
         <v>25</v>
       </c>
@@ -1921,6 +2632,620 @@
       </c>
       <c r="K2" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="102" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J3" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="119" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="204" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="68" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J6" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="119" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J7" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="51" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="119" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J9" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="68" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J10" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="119" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J11" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="102" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J12" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M12" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="102" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J13" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="68" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J14" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="68" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J15" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M15" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="51" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J16" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L16" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M16" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="119" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J17" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L17" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M17" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="34" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J18" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L18" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M18" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="34" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J19" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L19" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M19" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="34" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J20" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L20" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M20" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="34" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J21" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M21" s="1" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
puma review and some updates
</commit_message>
<xml_diff>
--- a/data/input/puma.xlsx
+++ b/data/input/puma.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Saowalak/Desktop/CEOCommunication/data/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1EC71AB-7B05-0F49-AE66-B4BEBF1638CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE43DD4-3883-4C46-819C-C3B428421F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="23780" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16720" yWindow="600" windowWidth="21660" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1276" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1407" uniqueCount="251">
   <si>
     <t>ID</t>
   </si>
@@ -655,9 +655,6 @@
     <t>DEU25P00-00</t>
   </si>
   <si>
-    <t xml:space="preserve">False </t>
-  </si>
-  <si>
     <t>Arthur Hoeld</t>
   </si>
   <si>
@@ -755,7 +752,37 @@
     <t>Leadership_context_human</t>
   </si>
   <si>
-    <t>True</t>
+    <t>false</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>Salutation addressed to shareholders, although it contains no substantive information.</t>
+  </si>
+  <si>
+    <t>CHALL primary becuase it describes the disruption caused by store closures and the operational adaptation toward e-commerce, marketing, and logistics. MARKET is an alternative because channels and distribution are discussed;</t>
+  </si>
+  <si>
+    <t>Expresses appreciation for the supervisory board’s trust and support as an external governance stakeholder. The investments are context, not the primary communicative purpose.</t>
+  </si>
+  <si>
+    <t>CHALL primary because the passage focuses on COVID-related factory closures, supply-chain disruption, and production suspension. MARKET as an alternative because product supply is affected.</t>
+  </si>
+  <si>
+    <t>STAKE primary because it  focuses on equality, anti-discrimination, environmental sustainability, circularity, climate action, and social responsibility.</t>
+  </si>
+  <si>
+    <t>PERF primary because it reports realized product and commercial achievements. MARKET is an alternative because products and consumers are discussed, but achieved results dominate.</t>
+  </si>
+  <si>
+    <t>Closing goodwill and health message addressed to the PUMA audience, followed by the CEO signature. No substantive business context.</t>
+  </si>
+  <si>
+    <t>CEO signature. No substantive business context.</t>
+  </si>
+  <si>
+    <t>PERF is primary because the passage opens with realized 2020 business performance. MARKET is an alternative because consumer and sports-market trends are also discussed. CHALL is only background context.</t>
   </si>
 </sst>
 </file>
@@ -1123,6 +1150,8 @@
   <dimension ref="A1:P106"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="54" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" customWidth="1"/>
     <col min="4" max="4" width="11.6640625" customWidth="1"/>
     <col min="5" max="5" width="25.33203125" customWidth="1"/>
@@ -1148,7 +1177,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -1201,7 +1230,7 @@
         <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F2" t="s">
         <v>20</v>
@@ -1226,6 +1255,12 @@
       </c>
       <c r="M2" t="s">
         <v>25</v>
+      </c>
+      <c r="N2" t="s">
+        <v>242</v>
+      </c>
+      <c r="O2" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
@@ -1268,6 +1303,9 @@
       <c r="M3" t="s">
         <v>25</v>
       </c>
+      <c r="O3" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -1309,6 +1347,9 @@
       <c r="M4" t="s">
         <v>25</v>
       </c>
+      <c r="O4" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -1350,6 +1391,9 @@
       <c r="M5" t="s">
         <v>25</v>
       </c>
+      <c r="O5" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -1391,6 +1435,9 @@
       <c r="M6" t="s">
         <v>25</v>
       </c>
+      <c r="O6" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -1406,7 +1453,7 @@
         <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F7" t="s">
         <v>20</v>
@@ -1431,6 +1478,9 @@
       </c>
       <c r="M7" t="s">
         <v>25</v>
+      </c>
+      <c r="O7" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
@@ -1473,6 +1523,9 @@
       <c r="M8" t="s">
         <v>25</v>
       </c>
+      <c r="O8" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -1485,10 +1538,10 @@
         <v>28</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="E9" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F9" t="s">
         <v>20</v>
@@ -1513,6 +1566,9 @@
       </c>
       <c r="M9" t="s">
         <v>25</v>
+      </c>
+      <c r="O9" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
@@ -1555,6 +1611,9 @@
       <c r="M10" t="s">
         <v>25</v>
       </c>
+      <c r="O10" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -1567,7 +1626,7 @@
         <v>28</v>
       </c>
       <c r="D11" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="E11" t="s">
         <v>19</v>
@@ -1595,6 +1654,9 @@
       </c>
       <c r="M11" t="s">
         <v>25</v>
+      </c>
+      <c r="O11" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
@@ -1637,6 +1699,15 @@
       <c r="M12" t="s">
         <v>25</v>
       </c>
+      <c r="N12" t="s">
+        <v>243</v>
+      </c>
+      <c r="O12" t="s">
+        <v>241</v>
+      </c>
+      <c r="P12" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -1649,7 +1720,7 @@
         <v>28</v>
       </c>
       <c r="D13" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E13" t="s">
         <v>19</v>
@@ -1677,6 +1748,9 @@
       </c>
       <c r="M13" t="s">
         <v>25</v>
+      </c>
+      <c r="O13" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
@@ -1719,6 +1793,12 @@
       <c r="M14" t="s">
         <v>25</v>
       </c>
+      <c r="N14" t="s">
+        <v>244</v>
+      </c>
+      <c r="O14" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -1760,6 +1840,9 @@
       <c r="M15" t="s">
         <v>25</v>
       </c>
+      <c r="O15" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -1801,8 +1884,11 @@
       <c r="M16" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O16" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>63</v>
       </c>
@@ -1813,10 +1899,10 @@
         <v>28</v>
       </c>
       <c r="D17" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="E17" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F17" t="s">
         <v>20</v>
@@ -1842,8 +1928,17 @@
       <c r="M17" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N17" t="s">
+        <v>250</v>
+      </c>
+      <c r="O17" t="s">
+        <v>241</v>
+      </c>
+      <c r="P17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>65</v>
       </c>
@@ -1883,8 +1978,11 @@
       <c r="M18" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O18" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>67</v>
       </c>
@@ -1924,8 +2022,11 @@
       <c r="M19" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O19" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>69</v>
       </c>
@@ -1965,8 +2066,14 @@
       <c r="M20" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N20" t="s">
+        <v>248</v>
+      </c>
+      <c r="O20" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>71</v>
       </c>
@@ -1980,7 +2087,7 @@
         <v>18</v>
       </c>
       <c r="E21" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F21" t="s">
         <v>20</v>
@@ -2006,8 +2113,14 @@
       <c r="M21" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N21" t="s">
+        <v>242</v>
+      </c>
+      <c r="O21" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>72</v>
       </c>
@@ -2047,8 +2160,11 @@
       <c r="M22" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O22" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -2088,8 +2204,11 @@
       <c r="M23" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O23" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>76</v>
       </c>
@@ -2129,8 +2248,11 @@
       <c r="M24" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O24" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>78</v>
       </c>
@@ -2170,8 +2292,11 @@
       <c r="M25" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O25" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>80</v>
       </c>
@@ -2211,8 +2336,11 @@
       <c r="M26" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O26" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>82</v>
       </c>
@@ -2252,8 +2380,11 @@
       <c r="M27" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O27" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>84</v>
       </c>
@@ -2264,10 +2395,10 @@
         <v>28</v>
       </c>
       <c r="D28" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E28" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F28" t="s">
         <v>20</v>
@@ -2293,8 +2424,17 @@
       <c r="M28" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N28" t="s">
+        <v>245</v>
+      </c>
+      <c r="O28" t="s">
+        <v>241</v>
+      </c>
+      <c r="P28" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>86</v>
       </c>
@@ -2334,8 +2474,11 @@
       <c r="M29" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O29" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>88</v>
       </c>
@@ -2375,8 +2518,11 @@
       <c r="M30" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O30" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>90</v>
       </c>
@@ -2416,8 +2562,11 @@
       <c r="M31" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O31" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>92</v>
       </c>
@@ -2457,8 +2606,11 @@
       <c r="M32" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O32" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>94</v>
       </c>
@@ -2469,7 +2621,7 @@
         <v>28</v>
       </c>
       <c r="D33" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="E33" t="s">
         <v>19</v>
@@ -2498,8 +2650,14 @@
       <c r="M33" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N33" t="s">
+        <v>246</v>
+      </c>
+      <c r="O33" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>96</v>
       </c>
@@ -2539,8 +2697,11 @@
       <c r="M34" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O34" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>98</v>
       </c>
@@ -2551,10 +2712,10 @@
         <v>28</v>
       </c>
       <c r="D35" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="E35" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F35" t="s">
         <v>20</v>
@@ -2580,8 +2741,11 @@
       <c r="M35" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O35" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>100</v>
       </c>
@@ -2592,7 +2756,7 @@
         <v>28</v>
       </c>
       <c r="D36" t="s">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="E36" t="s">
         <v>37</v>
@@ -2621,8 +2785,14 @@
       <c r="M36" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N36" t="s">
+        <v>248</v>
+      </c>
+      <c r="O36" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>102</v>
       </c>
@@ -2636,7 +2806,7 @@
         <v>18</v>
       </c>
       <c r="E37" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F37" t="s">
         <v>20</v>
@@ -2662,8 +2832,14 @@
       <c r="M37" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N37" t="s">
+        <v>242</v>
+      </c>
+      <c r="O37" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>104</v>
       </c>
@@ -2703,8 +2879,11 @@
       <c r="M38" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O38" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>106</v>
       </c>
@@ -2744,8 +2923,11 @@
       <c r="M39" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O39" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>108</v>
       </c>
@@ -2785,8 +2967,11 @@
       <c r="M40" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O40" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>110</v>
       </c>
@@ -2826,8 +3011,11 @@
       <c r="M41" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O41" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>112</v>
       </c>
@@ -2867,8 +3055,11 @@
       <c r="M42" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O42" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>114</v>
       </c>
@@ -2908,8 +3099,11 @@
       <c r="M43" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O43" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>116</v>
       </c>
@@ -2949,8 +3143,11 @@
       <c r="M44" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O44" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>118</v>
       </c>
@@ -2990,8 +3187,11 @@
       <c r="M45" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O45" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>120</v>
       </c>
@@ -3031,8 +3231,11 @@
       <c r="M46" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O46" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>122</v>
       </c>
@@ -3072,8 +3275,17 @@
       <c r="M47" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N47" t="s">
+        <v>247</v>
+      </c>
+      <c r="O47" t="s">
+        <v>241</v>
+      </c>
+      <c r="P47" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>124</v>
       </c>
@@ -3113,8 +3325,11 @@
       <c r="M48" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O48" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>126</v>
       </c>
@@ -3128,7 +3343,7 @@
         <v>33</v>
       </c>
       <c r="E49" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F49" t="s">
         <v>20</v>
@@ -3154,8 +3369,11 @@
       <c r="M49" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O49" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>128</v>
       </c>
@@ -3195,8 +3413,11 @@
       <c r="M50" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O50" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>130</v>
       </c>
@@ -3236,8 +3457,11 @@
       <c r="M51" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O51" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>132</v>
       </c>
@@ -3277,8 +3501,11 @@
       <c r="M52" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O52" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>134</v>
       </c>
@@ -3292,7 +3519,7 @@
         <v>36</v>
       </c>
       <c r="E53" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F53" t="s">
         <v>20</v>
@@ -3318,8 +3545,11 @@
       <c r="M53" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O53" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>136</v>
       </c>
@@ -3359,8 +3589,11 @@
       <c r="M54" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O54" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>138</v>
       </c>
@@ -3374,7 +3607,7 @@
         <v>49</v>
       </c>
       <c r="E55" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F55" t="s">
         <v>20</v>
@@ -3400,8 +3633,11 @@
       <c r="M55" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O55" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>140</v>
       </c>
@@ -3412,7 +3648,7 @@
         <v>28</v>
       </c>
       <c r="D56" t="s">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="E56" t="s">
         <v>37</v>
@@ -3441,8 +3677,14 @@
       <c r="M56" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N56" t="s">
+        <v>249</v>
+      </c>
+      <c r="O56" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>142</v>
       </c>
@@ -3456,7 +3698,7 @@
         <v>18</v>
       </c>
       <c r="E57" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F57" t="s">
         <v>20</v>
@@ -3482,8 +3724,14 @@
       <c r="M57" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N57" t="s">
+        <v>242</v>
+      </c>
+      <c r="O57" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>143</v>
       </c>
@@ -3523,8 +3771,11 @@
       <c r="M58" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O58" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>145</v>
       </c>
@@ -3538,7 +3789,7 @@
         <v>36</v>
       </c>
       <c r="E59" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F59" t="s">
         <v>20</v>
@@ -3564,8 +3815,11 @@
       <c r="M59" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O59" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>147</v>
       </c>
@@ -3579,7 +3833,7 @@
         <v>36</v>
       </c>
       <c r="E60" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F60" t="s">
         <v>20</v>
@@ -3605,8 +3859,14 @@
       <c r="M60" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O60" t="s">
+        <v>241</v>
+      </c>
+      <c r="P60" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="61" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>149</v>
       </c>
@@ -3620,7 +3880,7 @@
         <v>36</v>
       </c>
       <c r="E61" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F61" t="s">
         <v>20</v>
@@ -3646,8 +3906,14 @@
       <c r="M61" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O61" t="s">
+        <v>241</v>
+      </c>
+      <c r="P61" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>151</v>
       </c>
@@ -3658,10 +3924,10 @@
         <v>28</v>
       </c>
       <c r="D62" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E62" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F62" t="s">
         <v>20</v>
@@ -3687,8 +3953,11 @@
       <c r="M62" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O62" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>153</v>
       </c>
@@ -3728,8 +3997,11 @@
       <c r="M63" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O63" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="64" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>155</v>
       </c>
@@ -3769,8 +4041,11 @@
       <c r="M64" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O64" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>157</v>
       </c>
@@ -3810,8 +4085,11 @@
       <c r="M65" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O65" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="66" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>159</v>
       </c>
@@ -3851,8 +4129,11 @@
       <c r="M66" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O66" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="67" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>161</v>
       </c>
@@ -3892,8 +4173,11 @@
       <c r="M67" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O67" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="68" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>163</v>
       </c>
@@ -3904,10 +4188,10 @@
         <v>28</v>
       </c>
       <c r="D68" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E68" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F68" t="s">
         <v>20</v>
@@ -3933,8 +4217,11 @@
       <c r="M68" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O68" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>165</v>
       </c>
@@ -3948,7 +4235,7 @@
         <v>36</v>
       </c>
       <c r="E69" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F69" t="s">
         <v>20</v>
@@ -3974,8 +4261,11 @@
       <c r="M69" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O69" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>167</v>
       </c>
@@ -3986,7 +4276,7 @@
         <v>28</v>
       </c>
       <c r="D70" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E70" t="s">
         <v>19</v>
@@ -4015,8 +4305,11 @@
       <c r="M70" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O70" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>169</v>
       </c>
@@ -4056,8 +4349,11 @@
       <c r="M71" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O71" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="72" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>171</v>
       </c>
@@ -4097,8 +4393,11 @@
       <c r="M72" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O72" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="73" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>173</v>
       </c>
@@ -4138,8 +4437,11 @@
       <c r="M73" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O73" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="74" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>175</v>
       </c>
@@ -4179,8 +4481,11 @@
       <c r="M74" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O74" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="75" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>177</v>
       </c>
@@ -4220,8 +4525,11 @@
       <c r="M75" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O75" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="76" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>179</v>
       </c>
@@ -4261,8 +4569,11 @@
       <c r="M76" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O76" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="77" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>181</v>
       </c>
@@ -4302,8 +4613,11 @@
       <c r="M77" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O77" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="78" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>183</v>
       </c>
@@ -4343,8 +4657,11 @@
       <c r="M78" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O78" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="79" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>185</v>
       </c>
@@ -4355,7 +4672,7 @@
         <v>28</v>
       </c>
       <c r="D79" t="s">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="E79" t="s">
         <v>37</v>
@@ -4384,8 +4701,14 @@
       <c r="M79" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N79" t="s">
+        <v>249</v>
+      </c>
+      <c r="O79" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="80" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>187</v>
       </c>
@@ -4399,7 +4722,7 @@
         <v>18</v>
       </c>
       <c r="E80" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F80" t="s">
         <v>20</v>
@@ -4417,7 +4740,7 @@
         <v>2024</v>
       </c>
       <c r="K80" t="s">
-        <v>208</v>
+        <v>240</v>
       </c>
       <c r="L80" t="s">
         <v>24</v>
@@ -4425,8 +4748,14 @@
       <c r="M80" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N80" t="s">
+        <v>242</v>
+      </c>
+      <c r="O80" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="81" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>188</v>
       </c>
@@ -4458,7 +4787,7 @@
         <v>2024</v>
       </c>
       <c r="K81" t="s">
-        <v>208</v>
+        <v>240</v>
       </c>
       <c r="L81" t="s">
         <v>24</v>
@@ -4466,8 +4795,11 @@
       <c r="M81" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O81" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="82" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>190</v>
       </c>
@@ -4499,7 +4831,7 @@
         <v>2024</v>
       </c>
       <c r="K82" t="s">
-        <v>208</v>
+        <v>240</v>
       </c>
       <c r="L82" t="s">
         <v>24</v>
@@ -4507,8 +4839,11 @@
       <c r="M82" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O82" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="83" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>192</v>
       </c>
@@ -4519,7 +4854,7 @@
         <v>28</v>
       </c>
       <c r="D83" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E83" t="s">
         <v>19</v>
@@ -4540,7 +4875,7 @@
         <v>2024</v>
       </c>
       <c r="K83" t="s">
-        <v>208</v>
+        <v>240</v>
       </c>
       <c r="L83" t="s">
         <v>24</v>
@@ -4548,8 +4883,14 @@
       <c r="M83" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O83" t="s">
+        <v>241</v>
+      </c>
+      <c r="P83" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="84" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>194</v>
       </c>
@@ -4581,7 +4922,7 @@
         <v>2024</v>
       </c>
       <c r="K84" t="s">
-        <v>208</v>
+        <v>240</v>
       </c>
       <c r="L84" t="s">
         <v>24</v>
@@ -4589,8 +4930,11 @@
       <c r="M84" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O84" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="85" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>196</v>
       </c>
@@ -4622,7 +4966,7 @@
         <v>2024</v>
       </c>
       <c r="K85" t="s">
-        <v>208</v>
+        <v>240</v>
       </c>
       <c r="L85" t="s">
         <v>24</v>
@@ -4630,8 +4974,11 @@
       <c r="M85" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O85" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="86" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>198</v>
       </c>
@@ -4642,7 +4989,7 @@
         <v>28</v>
       </c>
       <c r="D86" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E86" t="s">
         <v>19</v>
@@ -4663,7 +5010,7 @@
         <v>2024</v>
       </c>
       <c r="K86" t="s">
-        <v>208</v>
+        <v>240</v>
       </c>
       <c r="L86" t="s">
         <v>24</v>
@@ -4671,8 +5018,11 @@
       <c r="M86" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="87" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O86" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="87" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>200</v>
       </c>
@@ -4704,7 +5054,7 @@
         <v>2024</v>
       </c>
       <c r="K87" t="s">
-        <v>208</v>
+        <v>240</v>
       </c>
       <c r="L87" t="s">
         <v>24</v>
@@ -4712,8 +5062,11 @@
       <c r="M87" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O87" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="88" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>202</v>
       </c>
@@ -4745,7 +5098,7 @@
         <v>2024</v>
       </c>
       <c r="K88" t="s">
-        <v>208</v>
+        <v>240</v>
       </c>
       <c r="L88" t="s">
         <v>24</v>
@@ -4753,8 +5106,11 @@
       <c r="M88" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O88" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="89" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>204</v>
       </c>
@@ -4786,7 +5142,7 @@
         <v>2024</v>
       </c>
       <c r="K89" t="s">
-        <v>208</v>
+        <v>240</v>
       </c>
       <c r="L89" t="s">
         <v>24</v>
@@ -4794,8 +5150,11 @@
       <c r="M89" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O89" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="90" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>206</v>
       </c>
@@ -4806,7 +5165,7 @@
         <v>28</v>
       </c>
       <c r="D90" t="s">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="E90" t="s">
         <v>37</v>
@@ -4827,7 +5186,7 @@
         <v>2025</v>
       </c>
       <c r="K90" t="s">
-        <v>208</v>
+        <v>240</v>
       </c>
       <c r="L90" t="s">
         <v>24</v>
@@ -4835,8 +5194,14 @@
       <c r="M90" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N90" t="s">
+        <v>249</v>
+      </c>
+      <c r="O90" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="91" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>207</v>
       </c>
@@ -4850,7 +5215,7 @@
         <v>18</v>
       </c>
       <c r="E91" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F91" t="s">
         <v>20</v>
@@ -4868,21 +5233,27 @@
         <v>2025</v>
       </c>
       <c r="K91" t="s">
+        <v>240</v>
+      </c>
+      <c r="L91" t="s">
+        <v>24</v>
+      </c>
+      <c r="M91" t="s">
         <v>208</v>
       </c>
-      <c r="L91" t="s">
-        <v>24</v>
-      </c>
-      <c r="M91" t="s">
+      <c r="N91" t="s">
+        <v>242</v>
+      </c>
+      <c r="O91" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="92" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
+      <c r="B92" t="s">
         <v>210</v>
-      </c>
-      <c r="B92" t="s">
-        <v>211</v>
       </c>
       <c r="C92" t="s">
         <v>28</v>
@@ -4909,21 +5280,24 @@
         <v>2025</v>
       </c>
       <c r="K92" t="s">
+        <v>240</v>
+      </c>
+      <c r="L92" t="s">
+        <v>24</v>
+      </c>
+      <c r="M92" t="s">
         <v>208</v>
       </c>
-      <c r="L92" t="s">
-        <v>24</v>
-      </c>
-      <c r="M92" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O92" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="93" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
+        <v>211</v>
+      </c>
+      <c r="B93" t="s">
         <v>212</v>
-      </c>
-      <c r="B93" t="s">
-        <v>213</v>
       </c>
       <c r="C93" t="s">
         <v>28</v>
@@ -4950,21 +5324,24 @@
         <v>2025</v>
       </c>
       <c r="K93" t="s">
+        <v>240</v>
+      </c>
+      <c r="L93" t="s">
+        <v>24</v>
+      </c>
+      <c r="M93" t="s">
         <v>208</v>
       </c>
-      <c r="L93" t="s">
-        <v>24</v>
-      </c>
-      <c r="M93" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O93" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="94" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
+        <v>213</v>
+      </c>
+      <c r="B94" t="s">
         <v>214</v>
-      </c>
-      <c r="B94" t="s">
-        <v>215</v>
       </c>
       <c r="C94" t="s">
         <v>28</v>
@@ -4991,21 +5368,24 @@
         <v>2025</v>
       </c>
       <c r="K94" t="s">
+        <v>240</v>
+      </c>
+      <c r="L94" t="s">
+        <v>24</v>
+      </c>
+      <c r="M94" t="s">
         <v>208</v>
       </c>
-      <c r="L94" t="s">
-        <v>24</v>
-      </c>
-      <c r="M94" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O94" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="95" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
+        <v>215</v>
+      </c>
+      <c r="B95" t="s">
         <v>216</v>
-      </c>
-      <c r="B95" t="s">
-        <v>217</v>
       </c>
       <c r="C95" t="s">
         <v>28</v>
@@ -5032,21 +5412,24 @@
         <v>2025</v>
       </c>
       <c r="K95" t="s">
+        <v>240</v>
+      </c>
+      <c r="L95" t="s">
+        <v>24</v>
+      </c>
+      <c r="M95" t="s">
         <v>208</v>
       </c>
-      <c r="L95" t="s">
-        <v>24</v>
-      </c>
-      <c r="M95" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O95" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="96" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
+        <v>217</v>
+      </c>
+      <c r="B96" t="s">
         <v>218</v>
-      </c>
-      <c r="B96" t="s">
-        <v>219</v>
       </c>
       <c r="C96" t="s">
         <v>28</v>
@@ -5073,21 +5456,24 @@
         <v>2025</v>
       </c>
       <c r="K96" t="s">
+        <v>240</v>
+      </c>
+      <c r="L96" t="s">
+        <v>24</v>
+      </c>
+      <c r="M96" t="s">
         <v>208</v>
       </c>
-      <c r="L96" t="s">
-        <v>24</v>
-      </c>
-      <c r="M96" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O96" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="97" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
+        <v>219</v>
+      </c>
+      <c r="B97" t="s">
         <v>220</v>
-      </c>
-      <c r="B97" t="s">
-        <v>221</v>
       </c>
       <c r="C97" t="s">
         <v>28</v>
@@ -5114,21 +5500,24 @@
         <v>2025</v>
       </c>
       <c r="K97" t="s">
+        <v>240</v>
+      </c>
+      <c r="L97" t="s">
+        <v>24</v>
+      </c>
+      <c r="M97" t="s">
         <v>208</v>
       </c>
-      <c r="L97" t="s">
-        <v>24</v>
-      </c>
-      <c r="M97" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O97" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="98" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
+        <v>221</v>
+      </c>
+      <c r="B98" t="s">
         <v>222</v>
-      </c>
-      <c r="B98" t="s">
-        <v>223</v>
       </c>
       <c r="C98" t="s">
         <v>28</v>
@@ -5137,7 +5526,7 @@
         <v>36</v>
       </c>
       <c r="E98" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F98" t="s">
         <v>20</v>
@@ -5155,21 +5544,24 @@
         <v>2025</v>
       </c>
       <c r="K98" t="s">
+        <v>240</v>
+      </c>
+      <c r="L98" t="s">
+        <v>24</v>
+      </c>
+      <c r="M98" t="s">
         <v>208</v>
       </c>
-      <c r="L98" t="s">
-        <v>24</v>
-      </c>
-      <c r="M98" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O98" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="99" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
+        <v>223</v>
+      </c>
+      <c r="B99" t="s">
         <v>224</v>
-      </c>
-      <c r="B99" t="s">
-        <v>225</v>
       </c>
       <c r="C99" t="s">
         <v>28</v>
@@ -5178,7 +5570,7 @@
         <v>36</v>
       </c>
       <c r="E99" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F99" t="s">
         <v>20</v>
@@ -5196,21 +5588,24 @@
         <v>2025</v>
       </c>
       <c r="K99" t="s">
+        <v>240</v>
+      </c>
+      <c r="L99" t="s">
+        <v>24</v>
+      </c>
+      <c r="M99" t="s">
         <v>208</v>
       </c>
-      <c r="L99" t="s">
-        <v>24</v>
-      </c>
-      <c r="M99" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O99" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="100" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
+        <v>225</v>
+      </c>
+      <c r="B100" t="s">
         <v>226</v>
-      </c>
-      <c r="B100" t="s">
-        <v>227</v>
       </c>
       <c r="C100" t="s">
         <v>28</v>
@@ -5219,7 +5614,7 @@
         <v>36</v>
       </c>
       <c r="E100" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F100" t="s">
         <v>20</v>
@@ -5237,21 +5632,27 @@
         <v>2025</v>
       </c>
       <c r="K100" t="s">
+        <v>240</v>
+      </c>
+      <c r="L100" t="s">
+        <v>24</v>
+      </c>
+      <c r="M100" t="s">
         <v>208</v>
       </c>
-      <c r="L100" t="s">
-        <v>24</v>
-      </c>
-      <c r="M100" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O100" t="s">
+        <v>241</v>
+      </c>
+      <c r="P100" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="101" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
+        <v>227</v>
+      </c>
+      <c r="B101" t="s">
         <v>228</v>
-      </c>
-      <c r="B101" t="s">
-        <v>229</v>
       </c>
       <c r="C101" t="s">
         <v>28</v>
@@ -5260,7 +5661,7 @@
         <v>36</v>
       </c>
       <c r="E101" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F101" t="s">
         <v>20</v>
@@ -5278,21 +5679,24 @@
         <v>2025</v>
       </c>
       <c r="K101" t="s">
+        <v>240</v>
+      </c>
+      <c r="L101" t="s">
+        <v>24</v>
+      </c>
+      <c r="M101" t="s">
         <v>208</v>
       </c>
-      <c r="L101" t="s">
-        <v>24</v>
-      </c>
-      <c r="M101" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O101" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="102" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
+        <v>229</v>
+      </c>
+      <c r="B102" t="s">
         <v>230</v>
-      </c>
-      <c r="B102" t="s">
-        <v>231</v>
       </c>
       <c r="C102" t="s">
         <v>28</v>
@@ -5319,21 +5723,24 @@
         <v>2025</v>
       </c>
       <c r="K102" t="s">
+        <v>240</v>
+      </c>
+      <c r="L102" t="s">
+        <v>24</v>
+      </c>
+      <c r="M102" t="s">
         <v>208</v>
       </c>
-      <c r="L102" t="s">
-        <v>24</v>
-      </c>
-      <c r="M102" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O102" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="103" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
+        <v>231</v>
+      </c>
+      <c r="B103" t="s">
         <v>232</v>
-      </c>
-      <c r="B103" t="s">
-        <v>233</v>
       </c>
       <c r="C103" t="s">
         <v>28</v>
@@ -5360,21 +5767,24 @@
         <v>2025</v>
       </c>
       <c r="K103" t="s">
+        <v>240</v>
+      </c>
+      <c r="L103" t="s">
+        <v>24</v>
+      </c>
+      <c r="M103" t="s">
         <v>208</v>
       </c>
-      <c r="L103" t="s">
-        <v>24</v>
-      </c>
-      <c r="M103" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O103" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="104" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
+        <v>233</v>
+      </c>
+      <c r="B104" t="s">
         <v>234</v>
-      </c>
-      <c r="B104" t="s">
-        <v>235</v>
       </c>
       <c r="C104" t="s">
         <v>28</v>
@@ -5401,21 +5811,24 @@
         <v>2025</v>
       </c>
       <c r="K104" t="s">
+        <v>240</v>
+      </c>
+      <c r="L104" t="s">
+        <v>24</v>
+      </c>
+      <c r="M104" t="s">
         <v>208</v>
       </c>
-      <c r="L104" t="s">
-        <v>24</v>
-      </c>
-      <c r="M104" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O104" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="105" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
+        <v>235</v>
+      </c>
+      <c r="B105" t="s">
         <v>236</v>
-      </c>
-      <c r="B105" t="s">
-        <v>237</v>
       </c>
       <c r="C105" t="s">
         <v>28</v>
@@ -5442,27 +5855,30 @@
         <v>2025</v>
       </c>
       <c r="K105" t="s">
+        <v>240</v>
+      </c>
+      <c r="L105" t="s">
+        <v>24</v>
+      </c>
+      <c r="M105" t="s">
         <v>208</v>
       </c>
-      <c r="L105" t="s">
-        <v>24</v>
-      </c>
-      <c r="M105" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="106" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O105" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="106" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
+        <v>237</v>
+      </c>
+      <c r="B106" t="s">
         <v>238</v>
       </c>
-      <c r="B106" t="s">
-        <v>239</v>
-      </c>
       <c r="C106" t="s">
         <v>28</v>
       </c>
       <c r="D106" t="s">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="E106" t="s">
         <v>37</v>
@@ -5483,13 +5899,19 @@
         <v>2025</v>
       </c>
       <c r="K106" t="s">
+        <v>240</v>
+      </c>
+      <c r="L106" t="s">
+        <v>24</v>
+      </c>
+      <c r="M106" t="s">
         <v>208</v>
       </c>
-      <c r="L106" t="s">
-        <v>24</v>
-      </c>
-      <c r="M106" t="s">
-        <v>209</v>
+      <c r="N106" t="s">
+        <v>249</v>
+      </c>
+      <c r="O106" t="s">
+        <v>240</v>
       </c>
     </row>
   </sheetData>

</xml_diff>